<commit_message>
optimized backward even worse in e2e but better when compare individual kernel
</commit_message>
<xml_diff>
--- a/comprehensive_analysis_gs64_no_lora_360m.xlsx
+++ b/comprehensive_analysis_gs64_no_lora_360m.xlsx
@@ -62,14 +62,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -635,7 +635,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>compile_no_lora_360m</t>
+          <t>cuda_no_lora_360m_bwd_opt</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -652,16 +652,16 @@
         <v>2.069916248321533</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>2.295390605926514</v>
+        <v>1.254305362701416</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>-0.1089292176858917</v>
+        <v>0.3940308629788692</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>compile_no_lora_360m</t>
+          <t>cuda_no_lora_360m_bwd_opt</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -678,16 +678,16 @@
         <v>2.222823619842529</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>2.014636516571045</v>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>0.0936588496779753</v>
+        <v>0.8395440578460693</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>0.622307388516258</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>compile_no_lora_360m</t>
+          <t>cuda_no_lora_360m_bwd_opt</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -704,16 +704,16 @@
         <v>2.121335029602051</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>2.442120552062988</v>
+        <v>1.230266571044922</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>-0.1512186985952496</v>
+        <v>0.4200507916584433</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>compile_no_lora_360m</t>
+          <t>cuda_no_lora_360m_bwd_opt</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -730,16 +730,16 @@
         <v>2.122696876525879</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>1.856728792190552</v>
-      </c>
-      <c r="F11" s="5" t="n">
-        <v>0.1252972514712627</v>
+        <v>0.8926413059234619</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>0.5794777314675248</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>triton_no</t>
+          <t>compile_no_lora_360m</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -756,16 +756,16 @@
         <v>2.069916248321533</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2.160919666290283</v>
-      </c>
-      <c r="F12" s="4" t="n">
-        <v>-0.04396478265366699</v>
+        <v>2.295390605926514</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>-0.1089292176858917</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>triton_no</t>
+          <t>compile_no_lora_360m</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -782,16 +782,16 @@
         <v>2.222823619842529</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>2.164241552352905</v>
-      </c>
-      <c r="F13" s="5" t="n">
-        <v>0.02635479799957053</v>
+        <v>2.014636516571045</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>0.0936588496779753</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>triton_no</t>
+          <t>compile_no_lora_360m</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -808,16 +808,16 @@
         <v>2.121335029602051</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>2.128689289093018</v>
-      </c>
-      <c r="F14" s="4" t="n">
-        <v>-0.003466807170174534</v>
+        <v>2.442120552062988</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>-0.1512186985952496</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>triton_no</t>
+          <t>compile_no_lora_360m</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -834,16 +834,16 @@
         <v>2.122696876525879</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>1.930515050888061</v>
-      </c>
-      <c r="F15" s="5" t="n">
-        <v>0.09053663184936364</v>
+        <v>1.856728792190552</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>0.1252972514712627</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>cuda_no_lora_360m</t>
+          <t>triton_no</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -860,16 +860,16 @@
         <v>2.069916248321533</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>0.6602330207824707</v>
+        <v>2.160919666290283</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.6810339445773013</v>
+        <v>-0.04396478265366699</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>cuda_no_lora_360m</t>
+          <t>triton_no</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -886,16 +886,16 @@
         <v>2.222823619842529</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>1.056910276412964</v>
-      </c>
-      <c r="F17" s="5" t="n">
-        <v>0.5245190545132689</v>
+        <v>2.164241552352905</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>0.02635479799957053</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>cuda_no_lora_360m</t>
+          <t>triton_no</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -912,16 +912,16 @@
         <v>2.121335029602051</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>0.7126688957214355</v>
+        <v>2.128689289093018</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>0.6640469865549112</v>
+        <v>-0.003466807170174534</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>cuda_no_lora_360m</t>
+          <t>triton_no</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -938,10 +938,10 @@
         <v>2.122696876525879</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>0.786644458770752</v>
-      </c>
-      <c r="F19" s="5" t="n">
-        <v>0.6294127213970291</v>
+        <v>1.930515050888061</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>0.09053663184936364</v>
       </c>
     </row>
   </sheetData>
@@ -1132,7 +1132,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>compile_no_lora_360m</t>
+          <t>cuda_no_lora_360m_bwd_opt</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1149,16 +1149,16 @@
         <v>2.718506813049316</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>2.669891357421875</v>
-      </c>
-      <c r="F8" s="5" t="n">
-        <v>0.01788314651045882</v>
+        <v>1.360885143280029</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>0.4993997672738805</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>compile_no_lora_360m</t>
+          <t>cuda_no_lora_360m_bwd_opt</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1175,16 +1175,16 @@
         <v>3.014318227767944</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>2.571879863739014</v>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>0.1467789166894132</v>
+        <v>0.7596487998962402</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>0.747986528795021</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>compile_no_lora_360m</t>
+          <t>cuda_no_lora_360m_bwd_opt</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1201,16 +1201,16 @@
         <v>2.508376598358154</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>2.922121047973633</v>
+        <v>1.249581813812256</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>-0.1649451082769202</v>
+        <v>0.501836440895612</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>compile_no_lora_360m</t>
+          <t>cuda_no_lora_360m_bwd_opt</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1227,16 +1227,16 @@
         <v>2.515347242355347</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>2.001346826553345</v>
-      </c>
-      <c r="F11" s="5" t="n">
-        <v>0.2043457090722381</v>
+        <v>0.8353455066680908</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>0.6679005218039473</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>triton_no</t>
+          <t>compile_no_lora_360m</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1253,16 +1253,16 @@
         <v>2.718506813049316</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2.298252582550049</v>
-      </c>
-      <c r="F12" s="5" t="n">
-        <v>0.1545900964757463</v>
+        <v>2.669891357421875</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>0.01788314651045882</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>triton_no</t>
+          <t>compile_no_lora_360m</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1279,16 +1279,16 @@
         <v>3.014318227767944</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>2.294384241104126</v>
-      </c>
-      <c r="F13" s="5" t="n">
-        <v>0.2388380828645681</v>
+        <v>2.571879863739014</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>0.1467789166894132</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>triton_no</t>
+          <t>compile_no_lora_360m</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1305,16 +1305,16 @@
         <v>2.508376598358154</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>2.278536319732666</v>
+        <v>2.922121047973633</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.09162909539816673</v>
+        <v>-0.1649451082769202</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>triton_no</t>
+          <t>compile_no_lora_360m</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1331,16 +1331,16 @@
         <v>2.515347242355347</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>1.928260564804077</v>
-      </c>
-      <c r="F15" s="5" t="n">
-        <v>0.233401841171451</v>
+        <v>2.001346826553345</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>0.2043457090722381</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>cuda_no_lora_360m</t>
+          <t>triton_no</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1357,16 +1357,16 @@
         <v>2.718506813049316</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>3.052669525146484</v>
+        <v>2.298252582550049</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>-0.1229214179244015</v>
+        <v>0.1545900964757463</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>cuda_no_lora_360m</t>
+          <t>triton_no</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1383,16 +1383,16 @@
         <v>3.014318227767944</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>0.9925665855407716</v>
-      </c>
-      <c r="F17" s="5" t="n">
-        <v>0.6707160589757135</v>
+        <v>2.294384241104126</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>0.2388380828645681</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>cuda_no_lora_360m</t>
+          <t>triton_no</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1409,16 +1409,16 @@
         <v>2.508376598358154</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>3.050755977630615</v>
+        <v>2.278536319732666</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>-0.2162272521707756</v>
+        <v>0.09162909539816673</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>cuda_no_lora_360m</t>
+          <t>triton_no</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1435,10 +1435,10 @@
         <v>2.515347242355347</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>1.370407819747925</v>
-      </c>
-      <c r="F19" s="5" t="n">
-        <v>0.4551814569885436</v>
+        <v>1.928260564804077</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>0.233401841171451</v>
       </c>
     </row>
   </sheetData>
@@ -1629,7 +1629,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>compile_no_lora_360m</t>
+          <t>cuda_no_lora_360m_bwd_opt</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1648,14 +1648,14 @@
       <c r="E8" s="3" t="n">
         <v>0.0195964813232421</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F8" s="4" t="n">
         <v>0.1941298277539011</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>compile_no_lora_360m</t>
+          <t>cuda_no_lora_360m_bwd_opt</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1674,14 +1674,14 @@
       <c r="E9" s="3" t="n">
         <v>0.0026344299316406</v>
       </c>
-      <c r="F9" s="5" t="n">
+      <c r="F9" s="4" t="n">
         <v>0.1830602708936967</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>compile_no_lora_360m</t>
+          <t>cuda_no_lora_360m_bwd_opt</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1698,16 +1698,16 @@
         <v>0.0248912811279296</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0.0239013442993164</v>
-      </c>
-      <c r="F10" s="5" t="n">
-        <v>0.03977042497432674</v>
+        <v>0.0201705932617187</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>0.1896522658656564</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>compile_no_lora_360m</t>
+          <t>cuda_no_lora_360m_bwd_opt</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1726,14 +1726,14 @@
       <c r="E11" s="3" t="n">
         <v>0.0072443008422851</v>
       </c>
-      <c r="F11" s="5" t="n">
+      <c r="F11" s="4" t="n">
         <v>0.2503148279006619</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>triton_no</t>
+          <t>compile_no_lora_360m</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1750,16 +1750,16 @@
         <v>0.0243171691894531</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.0195979118347167</v>
-      </c>
-      <c r="F12" s="5" t="n">
-        <v>0.1940710005333699</v>
+        <v>0.0195964813232421</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>0.1941298277539011</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>triton_no</t>
+          <t>compile_no_lora_360m</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1776,16 +1776,16 @@
         <v>0.003224754333496</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0.0026358604431152</v>
-      </c>
-      <c r="F13" s="5" t="n">
-        <v>0.1826166676524385</v>
+        <v>0.0026344299316406</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>0.1830602708936967</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>triton_no</t>
+          <t>compile_no_lora_360m</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1802,16 +1802,16 @@
         <v>0.0248912811279296</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>0.0201720237731933</v>
-      </c>
-      <c r="F14" s="5" t="n">
-        <v>0.1895947954820612</v>
+        <v>0.0239013442993164</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>0.03977042497432674</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>triton_no</t>
+          <t>compile_no_lora_360m</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1828,16 +1828,16 @@
         <v>0.009663124084472599</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>0.0072457313537597</v>
-      </c>
-      <c r="F15" s="5" t="n">
-        <v>0.25016678970286</v>
+        <v>0.0072443008422851</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>0.2503148279006619</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>cuda_no_lora_360m</t>
+          <t>triton_no</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1854,16 +1854,16 @@
         <v>0.0243171691894531</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>0.0195964813232421</v>
-      </c>
-      <c r="F16" s="5" t="n">
-        <v>0.1941298277539011</v>
+        <v>0.0195979118347167</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>0.1940710005333699</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>cuda_no_lora_360m</t>
+          <t>triton_no</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1880,16 +1880,16 @@
         <v>0.003224754333496</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>0.0026344299316406</v>
-      </c>
-      <c r="F17" s="5" t="n">
-        <v>0.1830602708936967</v>
+        <v>0.0026358604431152</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>0.1826166676524385</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>cuda_no_lora_360m</t>
+          <t>triton_no</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1906,16 +1906,16 @@
         <v>0.0248912811279296</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>0.0201705932617187</v>
-      </c>
-      <c r="F18" s="5" t="n">
-        <v>0.1896522658656564</v>
+        <v>0.0201720237731933</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>0.1895947954820612</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>cuda_no_lora_360m</t>
+          <t>triton_no</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1932,10 +1932,10 @@
         <v>0.009663124084472599</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>0.0072443008422851</v>
-      </c>
-      <c r="F19" s="5" t="n">
-        <v>0.2503148279006619</v>
+        <v>0.0072457313537597</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>0.25016678970286</v>
       </c>
     </row>
   </sheetData>
@@ -2126,7 +2126,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>compile_no_lora_360m</t>
+          <t>cuda_no_lora_360m_bwd_opt</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2143,16 +2143,16 @@
         <v>0.0559415817260742</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.0422086715698242</v>
-      </c>
-      <c r="F8" s="5" t="n">
-        <v>0.2454866260931827</v>
+        <v>0.0241127014160156</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>0.5689663990180537</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>compile_no_lora_360m</t>
+          <t>cuda_no_lora_360m_bwd_opt</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2169,16 +2169,16 @@
         <v>0.0071773529052734</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0.0054607391357421</v>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>0.2391708743024265</v>
+        <v>0.0031991004943847</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>0.5542785011958611</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>compile_no_lora_360m</t>
+          <t>cuda_no_lora_360m_bwd_opt</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2195,16 +2195,16 @@
         <v>0.0565156936645507</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0.0419341659545898</v>
-      </c>
-      <c r="F10" s="5" t="n">
-        <v>0.258008471001164</v>
+        <v>0.0246868133544921</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>0.5631865813941723</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>compile_no_lora_360m</t>
+          <t>cuda_no_lora_360m_bwd_opt</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2221,16 +2221,16 @@
         <v>0.0215210914611816</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0.0163712501525878</v>
-      </c>
-      <c r="F11" s="5" t="n">
-        <v>0.2392927569627573</v>
+        <v>0.008936882019042899</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>0.5847384397226001</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>triton_no</t>
+          <t>compile_no_lora_360m</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2247,16 +2247,16 @@
         <v>0.0559415817260742</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.0329837799072265</v>
-      </c>
-      <c r="F12" s="5" t="n">
-        <v>0.4103888576348054</v>
+        <v>0.0422086715698242</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>0.2454866260931827</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>triton_no</t>
+          <t>compile_no_lora_360m</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2273,16 +2273,16 @@
         <v>0.0071773529052734</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0.0043091773986816</v>
-      </c>
-      <c r="F13" s="5" t="n">
-        <v>0.3996146691469598</v>
+        <v>0.0054607391357421</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>0.2391708743024265</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>triton_no</t>
+          <t>compile_no_lora_360m</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2299,16 +2299,16 @@
         <v>0.0565156936645507</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>0.0335578918457031</v>
-      </c>
-      <c r="F14" s="5" t="n">
-        <v>0.4062199422891949</v>
+        <v>0.0419341659545898</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>0.258008471001164</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>triton_no</t>
+          <t>compile_no_lora_360m</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2325,16 +2325,16 @@
         <v>0.0215210914611816</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>0.0122642517089843</v>
-      </c>
-      <c r="F15" s="5" t="n">
-        <v>0.4301287306405536</v>
+        <v>0.0163712501525878</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>0.2392927569627573</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>cuda_no_lora_360m</t>
+          <t>triton_no</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2351,16 +2351,16 @@
         <v>0.0559415817260742</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>0.0244703292846679</v>
-      </c>
-      <c r="F16" s="5" t="n">
-        <v>0.5625735181302113</v>
+        <v>0.0329837799072265</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>0.4103888576348054</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>cuda_no_lora_360m</t>
+          <t>triton_no</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2377,16 +2377,16 @@
         <v>0.0071773529052734</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>0.003244400024414</v>
-      </c>
-      <c r="F17" s="5" t="n">
-        <v>0.5479670475684358</v>
+        <v>0.0043091773986816</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>0.3996146691469598</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>cuda_no_lora_360m</t>
+          <t>triton_no</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2403,16 +2403,16 @@
         <v>0.0565156936645507</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>0.0250444412231445</v>
-      </c>
-      <c r="F18" s="5" t="n">
-        <v>0.5568586422773829</v>
+        <v>0.0335578918457031</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>0.4062199422891949</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>cuda_no_lora_360m</t>
+          <t>triton_no</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2429,10 +2429,10 @@
         <v>0.0215210914611816</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>0.009071826934814399</v>
-      </c>
-      <c r="F19" s="5" t="n">
-        <v>0.578468083220705</v>
+        <v>0.0122642517089843</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>0.4301287306405536</v>
       </c>
     </row>
   </sheetData>

</xml_diff>